<commit_message>
Alterações realizadas no arquivo conversor.py para gerar o 'tudd' corretamente além de melhorias na saída de dados do modelo 2 para melhor visualização.
</commit_message>
<xml_diff>
--- a/codigos_estudo/planilhas_xlsx/planilha_entrada_v1.xlsx
+++ b/codigos_estudo/planilhas_xlsx/planilha_entrada_v1.xlsx
@@ -64,7 +64,7 @@
     <t xml:space="preserve">hi</t>
   </si>
   <si>
-    <t xml:space="preserve">2 2 2 2 2 3 3 3 3 3 3 4 4 4</t>
+    <t xml:space="preserve">4 4 1 1 3 3 2 4</t>
   </si>
   <si>
     <t xml:space="preserve">ij</t>
@@ -73,13 +73,13 @@
     <t xml:space="preserve">vector_in_vector</t>
   </si>
   <si>
-    <t xml:space="preserve">1 2 6 7;1 8 9 10;5 13 14;3 4 11 12</t>
+    <t xml:space="preserve">1 2;3 4;5 6 7;8</t>
   </si>
   <si>
     <t xml:space="preserve">ig</t>
   </si>
   <si>
-    <t xml:space="preserve">1 2 3 6 7 12 13;4 5 8 9 10 11 14</t>
+    <t xml:space="preserve">1 2 3 4;5 6 7 8;1 2 8</t>
   </si>
 </sst>
 </file>
@@ -154,7 +154,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -165,6 +165,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -317,8 +321,8 @@
       <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="1" t="n">
-        <v>20</v>
+      <c r="C2" s="3" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -328,8 +332,8 @@
       <c r="B3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="1" t="n">
-        <v>5</v>
+      <c r="C3" s="3" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -339,7 +343,7 @@
       <c r="B4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="1" t="n">
+      <c r="C4" s="3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -350,8 +354,8 @@
       <c r="B5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="1" t="n">
-        <v>2</v>
+      <c r="C5" s="3" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -361,8 +365,8 @@
       <c r="B6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="1" t="n">
-        <v>14</v>
+      <c r="C6" s="3" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -372,7 +376,7 @@
       <c r="B7" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="1" t="n">
+      <c r="C7" s="3" t="n">
         <v>4</v>
       </c>
     </row>
@@ -383,8 +387,8 @@
       <c r="B8" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="1" t="n">
-        <v>4</v>
+      <c r="C8" s="3" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -394,40 +398,40 @@
       <c r="B9" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="1" t="n">
+      <c r="C9" s="3" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="12.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="12.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="12.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
         <v>18</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" s="3" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Código do conversor com adição de conjuntos e subconjuntos, adição das novas restrições e variáveis ao modelo também
</commit_message>
<xml_diff>
--- a/codigos_estudo/planilhas_xlsx/planilha_entrada_v1.xlsx
+++ b/codigos_estudo/planilhas_xlsx/planilha_entrada_v1.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="27">
   <si>
     <t xml:space="preserve">NOME</t>
   </si>
@@ -80,6 +80,27 @@
   </si>
   <si>
     <t xml:space="preserve">1 2 3 4;5 6 7 8;1 2 8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ki</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 2;4 6;4;8;1;7;4 2;3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">qk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20 20 20 20 20 20 20 20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18 12 14 10 8 9 10 11</t>
   </si>
 </sst>
 </file>
@@ -167,7 +188,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -436,20 +457,48 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
+      <c r="A13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="1" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
+      <c r="A14" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
+      <c r="A15" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
+      <c r="A16" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2"/>
@@ -4436,13 +4485,21 @@
       <c r="B1012" s="2"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A2:A1012" type="list">
+  <dataValidations count="4">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A41:A1012" type="list">
       <formula1>t d sd p sdp g ij ig i j lmax np tud tpdd hi</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B2:B1012" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B2 B4:B1012" type="list">
       <formula1>scalar vector vector_in_vector matrix matrix_of_vector</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B3" type="list">
+      <formula1>scalar vector vector_in_vector matrix matrix_of_vector</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A2:A40" type="list">
+      <formula1>t d sd p sdp g ij ig i j lmax np tud tpdd hi vi ki qk k</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>